<commit_message>
feat: engine model master per brand, canonicalize compatibility and resolve
- Add EngineModel model and /api/engine-models CRUD (scoped to brand).
- Canonicalize brand + engineModel on compatibility create/update and import.
- Resolve API validates engine model against master.
- UI: Engine models page, compatibility modal uses brand id + model dropdown.
- Seed Wärtsilä demo models; update import template instructions.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/marivolt-erp/sample-templates/Import_Material_Compatibility.xlsx
+++ b/marivolt-erp/sample-templates/Import_Material_Compatibility.xlsx
@@ -478,7 +478,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <cols>
     <col min="1" max="1" width="110.83203125" customWidth="1"/>
   </cols>
@@ -510,32 +510,37 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Legacy column engineMake is accepted by the API as an alias for brand.</v>
+        <v>engineModel: must match an Active Engine model under that brand (Engine models master).</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>remarks: optional. Legacy applicabilityRemarks is also accepted.</v>
+        <v>Legacy column engineMake is accepted by the API as an alias for brand.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v>remarks: optional. Legacy applicabilityRemarks is also accepted.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>esnFrom / esnTo: optional numbers; leave blank if not used.</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>esnFrom / esnTo: optional numbers; leave blank if not used.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>Each row creates a new compatibility record; duplicate keys in DB will fail that row.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>